<commit_message>
Removed the use of torch in MMTO_obj_cons_sensitivity
</commit_message>
<xml_diff>
--- a/DataConstantTemperature/5MaterialsCantilever.xlsx
+++ b/DataConstantTemperature/5MaterialsCantilever.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\METALS\DataConstantTemperature\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Personal\suresh\Software\Github\ERSL-Private\METALS\DataConstantTemperature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CE56B0D-AE21-434B-AB23-FF59BCF94DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{240E9D2E-80A0-45D8-A491-28E5D5FF4CDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -514,14 +514,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" style="3" customWidth="1"/>
-    <col min="2" max="701" width="20.5703125" style="3" customWidth="1"/>
-    <col min="702" max="16384" width="9.140625" style="3"/>
+    <col min="1" max="1" width="20.6640625" style="3" customWidth="1"/>
+    <col min="2" max="701" width="20.5546875" style="3" customWidth="1"/>
+    <col min="702" max="16384" width="9.109375" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>17</v>
       </c>
@@ -532,7 +532,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>18</v>
       </c>
@@ -543,7 +543,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>19</v>
       </c>
@@ -554,7 +554,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>20</v>
       </c>
@@ -565,7 +565,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>21</v>
       </c>
@@ -576,7 +576,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>22</v>
       </c>
@@ -587,7 +587,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
         <v>23</v>
       </c>
@@ -623,12 +623,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECC80EBF-8B96-4896-8C13-AD8A976D05A3}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -642,7 +642,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -656,7 +656,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -670,7 +670,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -684,7 +684,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>

</xml_diff>